<commit_message>
docs(governance): roadmap-review 2026-10-09 — idle-period pass + BUG-184 queued
No commits since 2026-07-03 (last code 2026-06-01). Buffer re-verified:
all 5 queued full specs still dispatch-ready, edit sites unchanged on main.

- Queue BUG-184 (filed 2026-05-29, never queued) as HOTFIX-EINK-HOVER-1 at
  Seq 6 with a full spec. Root cause widened: the wildcard
  [data-eink="true"] *:hover rule also matches hovered ancestors, so every
  background-bearing panel/dialog goes transparent, not just Settings.
  Reproduced and fix verified in headless Chromium.
- Correct CLAUDE.md Current System State (was 4 sprints stale and named
  the already-completed PAUSE-RESUME-UNIFY-1 as next dispatch).
- ROADMAP header/frontmatter + Catalog row + Dashboard queue cells.
- Review artifact: docs/planning/roadmap-reviews/2026-10-09-review.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VKGuAZ7hRqiqnBXZ1bsYH8
</commit_message>
<xml_diff>
--- a/docs/governance/sprint-queue.xlsx
+++ b/docs/governance/sprint-queue.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:H8"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="3" customWidth="1" style="12" min="1" max="1"/>
@@ -516,6 +516,7 @@
         <v>35</v>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="15" customHeight="1" s="12">
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -535,7 +536,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -543,7 +544,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -584,7 +585,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
@@ -603,7 +604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O53"/>
+  <dimension ref="A1:O54"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" style="12" min="1" max="1"/>
@@ -3915,6 +3916,61 @@
         </is>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>6</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>HOTFIX-EINK-HOVER-1</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Scope e-ink no-hover rule so panels/dialogs keep their background (BUG-184)</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Reader Runtime Solidification</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Active Conveyor Belt</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Queued</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Full Spec</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>Replace wildcard [data-eink="true"] *:hover {background-color: inherit} (themes.css:145) with an :is() list of the elements that carry a hover background; the wildcard also matches hovered ancestors and turns Settings flap, command palette and modals transparent.</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>sprint/hotfix-eink-hover-1</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>BUG-184 filed 2026-05-29, queued 2026-10-09 roadmap-review. Lane C, CSS-only, parallel-safe.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>